<commit_message>
#53 Client BOM Update
J11 ko update kia ha 6 Pin connector se
</commit_message>
<xml_diff>
--- a/Design Files/Powermodule-v11.0.0/Deliverables/BOM/Client-BOM-Powermodule-v11.0.0.xlsx
+++ b/Design Files/Powermodule-v11.0.0/Deliverables/BOM/Client-BOM-Powermodule-v11.0.0.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Iftikhar Ahmed\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\gerholdvoorde-dronebms\Design Files\Powermodule-v11.0.0\Deliverables\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -159,9 +159,6 @@
     <t>FB1</t>
   </si>
   <si>
-    <t>J1, J11</t>
-  </si>
-  <si>
     <t>J2</t>
   </si>
   <si>
@@ -180,9 +177,6 @@
     <t>J10</t>
   </si>
   <si>
-    <t>J12</t>
-  </si>
-  <si>
     <t>L1</t>
   </si>
   <si>
@@ -1090,6 +1084,12 @@
   </si>
   <si>
     <t>DO NOT PLACE</t>
+  </si>
+  <si>
+    <t>J11,J12</t>
+  </si>
+  <si>
+    <t>J1</t>
   </si>
 </sst>
 </file>
@@ -1335,9 +1335,6 @@
     <xf numFmtId="11" fontId="4" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1358,6 +1355,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1670,9 +1670,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="16"/>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" thickBot="1">
       <c r="A2" s="1"/>
@@ -1686,25 +1686,25 @@
         <v>28</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="J2" s="5" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="36.75" thickBot="1">
@@ -1720,19 +1720,19 @@
         <v>29</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="I3" s="8" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="J3" s="7">
         <v>4</v>
@@ -1752,19 +1752,19 @@
         <v>30</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J4" s="9">
         <v>8</v>
@@ -1784,19 +1784,19 @@
         <v>31</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="J5" s="7">
         <v>20</v>
@@ -1816,19 +1816,19 @@
         <v>32</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="J6" s="9">
         <v>2</v>
@@ -1848,19 +1848,19 @@
         <v>33</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="J7" s="7">
         <v>6</v>
@@ -1880,19 +1880,19 @@
         <v>34</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="J8" s="9">
         <v>5</v>
@@ -1912,19 +1912,19 @@
         <v>35</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="I9" s="8" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J9" s="7">
         <v>2</v>
@@ -1944,19 +1944,19 @@
         <v>36</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="J10" s="9">
         <v>4</v>
@@ -1976,19 +1976,19 @@
         <v>37</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J11" s="7">
         <v>1</v>
@@ -2008,19 +2008,19 @@
         <v>38</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J12" s="9">
         <v>1</v>
@@ -2040,19 +2040,19 @@
         <v>39</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J13" s="7">
         <v>2</v>
@@ -2072,19 +2072,19 @@
         <v>40</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J14" s="9">
         <v>11</v>
@@ -2104,19 +2104,19 @@
         <v>41</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J15" s="7">
         <v>1</v>
@@ -2136,19 +2136,19 @@
         <v>42</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F16" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J16" s="9">
         <v>8</v>
@@ -2168,19 +2168,19 @@
         <v>43</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J17" s="7">
         <v>2</v>
@@ -2200,19 +2200,19 @@
         <v>44</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F18" s="9" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="H18" s="9" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
@@ -2232,19 +2232,19 @@
         <v>45</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J19" s="7">
         <v>1</v>
@@ -2261,25 +2261,25 @@
         <v>6</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>46</v>
+        <v>356</v>
       </c>
       <c r="E20" s="10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="I20" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J20" s="9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" s="9"/>
     </row>
@@ -2293,22 +2293,22 @@
         <v>7</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I21" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J21" s="7">
         <v>1</v>
@@ -2325,22 +2325,22 @@
         <v>7</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="I22" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J22" s="9">
         <v>1</v>
@@ -2357,22 +2357,22 @@
         <v>8</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F23" s="7" t="s">
         <v>8</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J23" s="7">
         <v>4</v>
@@ -2389,22 +2389,22 @@
         <v>9</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F24" s="14" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="H24" s="9" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J24" s="9">
         <v>1</v>
@@ -2421,22 +2421,22 @@
         <v>10</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="H25" s="7" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J25" s="7">
         <v>1</v>
@@ -2453,22 +2453,22 @@
         <v>11</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J26" s="9">
         <v>1</v>
@@ -2485,25 +2485,25 @@
         <v>12</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>53</v>
+        <v>355</v>
       </c>
       <c r="E27" s="8" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="H27" s="7" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="I27" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J27" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K27" s="7"/>
     </row>
@@ -2517,22 +2517,22 @@
         <v>13</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="I28" s="10" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="J28" s="9">
         <v>1</v>
@@ -2549,22 +2549,22 @@
         <v>13</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E29" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="H29" s="7" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="J29" s="7">
         <v>1</v>
@@ -2581,22 +2581,22 @@
         <v>14</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F30" s="9" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="H30" s="9" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="I30" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J30" s="9">
         <v>3</v>
@@ -2612,29 +2612,29 @@
       <c r="C31" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D31" s="22" t="s">
-        <v>57</v>
-      </c>
-      <c r="E31" s="23" t="s">
-        <v>134</v>
-      </c>
-      <c r="F31" s="22" t="s">
-        <v>198</v>
-      </c>
-      <c r="G31" s="23" t="s">
-        <v>242</v>
-      </c>
-      <c r="H31" s="22" t="s">
-        <v>298</v>
-      </c>
-      <c r="I31" s="23" t="s">
-        <v>329</v>
-      </c>
-      <c r="J31" s="22">
-        <v>1</v>
-      </c>
-      <c r="K31" s="21" t="s">
-        <v>356</v>
+      <c r="D31" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="E31" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="F31" s="21" t="s">
+        <v>196</v>
+      </c>
+      <c r="G31" s="22" t="s">
+        <v>240</v>
+      </c>
+      <c r="H31" s="21" t="s">
+        <v>296</v>
+      </c>
+      <c r="I31" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="J31" s="21">
+        <v>1</v>
+      </c>
+      <c r="K31" s="20" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="32" spans="1:11" ht="48.75" thickBot="1">
@@ -2647,20 +2647,20 @@
         <v>15</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="G32" s="10" t="s">
         <v>15</v>
       </c>
       <c r="H32" s="9"/>
       <c r="I32" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J32" s="9">
         <v>33</v>
@@ -2677,22 +2677,22 @@
         <v>18</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E33" s="8" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="F33" s="7" t="s">
         <v>16</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="I33" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J33" s="7">
         <v>1</v>
@@ -2709,22 +2709,22 @@
         <v>17</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F34" s="9" t="s">
         <v>16</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="H34" s="9" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="I34" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J34" s="9">
         <v>2</v>
@@ -2741,22 +2741,22 @@
         <v>18</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E35" s="8" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F35" s="7" t="s">
         <v>16</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="I35" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J35" s="7">
         <v>1</v>
@@ -2773,22 +2773,22 @@
         <v>19</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F36" s="9" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="H36" s="9" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="I36" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J36" s="9">
         <v>1</v>
@@ -2804,29 +2804,29 @@
       <c r="C37" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D37" s="22" t="s">
-        <v>63</v>
-      </c>
-      <c r="E37" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="F37" s="22" t="s">
-        <v>201</v>
-      </c>
-      <c r="G37" s="23" t="s">
-        <v>247</v>
-      </c>
-      <c r="H37" s="22" t="s">
-        <v>289</v>
-      </c>
-      <c r="I37" s="23" t="s">
-        <v>329</v>
-      </c>
-      <c r="J37" s="22">
-        <v>1</v>
-      </c>
-      <c r="K37" s="21" t="s">
-        <v>356</v>
+      <c r="D37" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="E37" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="F37" s="21" t="s">
+        <v>199</v>
+      </c>
+      <c r="G37" s="22" t="s">
+        <v>245</v>
+      </c>
+      <c r="H37" s="21" t="s">
+        <v>287</v>
+      </c>
+      <c r="I37" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="J37" s="21">
+        <v>1</v>
+      </c>
+      <c r="K37" s="20" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="38" spans="1:11" ht="15.75" thickBot="1">
@@ -2839,22 +2839,22 @@
         <v>21</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="H38" s="9" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I38" s="10" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="J38" s="9">
         <v>1</v>
@@ -2871,22 +2871,22 @@
         <v>21</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E39" s="8" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="H39" s="7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I39" s="8" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="J39" s="7">
         <v>12</v>
@@ -2903,22 +2903,22 @@
         <v>21</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G40" s="10" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="H40" s="9" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I40" s="10" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J40" s="9">
         <v>1</v>
@@ -2935,22 +2935,22 @@
         <v>21</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E41" s="8" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H41" s="7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I41" s="8" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J41" s="7">
         <v>3</v>
@@ -2967,22 +2967,22 @@
         <v>21</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E42" s="10" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H42" s="9" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I42" s="10" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J42" s="9">
         <v>14</v>
@@ -2998,29 +2998,29 @@
       <c r="C43" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D43" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="E43" s="23" t="s">
-        <v>146</v>
-      </c>
-      <c r="F43" s="22" t="s">
-        <v>202</v>
-      </c>
-      <c r="G43" s="23" t="s">
-        <v>253</v>
-      </c>
-      <c r="H43" s="22" t="s">
-        <v>283</v>
-      </c>
-      <c r="I43" s="23" t="s">
-        <v>329</v>
-      </c>
-      <c r="J43" s="22">
-        <v>1</v>
-      </c>
-      <c r="K43" s="21" t="s">
-        <v>356</v>
+      <c r="D43" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="E43" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="F43" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="G43" s="22" t="s">
+        <v>251</v>
+      </c>
+      <c r="H43" s="21" t="s">
+        <v>281</v>
+      </c>
+      <c r="I43" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="J43" s="21">
+        <v>1</v>
+      </c>
+      <c r="K43" s="20" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="44" spans="1:11" ht="15.75" thickBot="1">
@@ -3033,22 +3033,22 @@
         <v>21</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E44" s="10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F44" s="9" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G44" s="10" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="H44" s="9" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="I44" s="10" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J44" s="9">
         <v>6</v>
@@ -3064,29 +3064,29 @@
       <c r="C45" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D45" s="22" t="s">
-        <v>71</v>
-      </c>
-      <c r="E45" s="23" t="s">
-        <v>145</v>
-      </c>
-      <c r="F45" s="22" t="s">
-        <v>202</v>
-      </c>
-      <c r="G45" s="23" t="s">
-        <v>252</v>
-      </c>
-      <c r="H45" s="22" t="s">
-        <v>283</v>
-      </c>
-      <c r="I45" s="23" t="s">
-        <v>329</v>
-      </c>
-      <c r="J45" s="22">
+      <c r="D45" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="E45" s="22" t="s">
+        <v>143</v>
+      </c>
+      <c r="F45" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="G45" s="22" t="s">
+        <v>250</v>
+      </c>
+      <c r="H45" s="21" t="s">
+        <v>281</v>
+      </c>
+      <c r="I45" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="J45" s="21">
         <v>3</v>
       </c>
-      <c r="K45" s="21" t="s">
-        <v>356</v>
+      <c r="K45" s="20" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="15.75" thickBot="1">
@@ -3099,22 +3099,22 @@
         <v>21</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E46" s="10" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F46" s="9" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G46" s="10" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="H46" s="9" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I46" s="10" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="J46" s="9">
         <v>3</v>
@@ -3131,22 +3131,22 @@
         <v>21</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E47" s="8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F47" s="7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="I47" s="8" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J47" s="7">
         <v>2</v>
@@ -3162,29 +3162,29 @@
       <c r="C48" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D48" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="E48" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="F48" s="22" t="s">
-        <v>202</v>
-      </c>
-      <c r="G48" s="23" t="s">
-        <v>255</v>
-      </c>
-      <c r="H48" s="22" t="s">
-        <v>283</v>
-      </c>
-      <c r="I48" s="23" t="s">
-        <v>329</v>
-      </c>
-      <c r="J48" s="22">
+      <c r="D48" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="E48" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="F48" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="G48" s="22" t="s">
+        <v>253</v>
+      </c>
+      <c r="H48" s="21" t="s">
+        <v>281</v>
+      </c>
+      <c r="I48" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="J48" s="21">
         <v>2</v>
       </c>
-      <c r="K48" s="21" t="s">
-        <v>356</v>
+      <c r="K48" s="20" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="49" spans="1:11" ht="15.75" thickBot="1">
@@ -3196,29 +3196,29 @@
       <c r="C49" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D49" s="22" t="s">
-        <v>75</v>
-      </c>
-      <c r="E49" s="23" t="s">
-        <v>150</v>
-      </c>
-      <c r="F49" s="22" t="s">
-        <v>202</v>
-      </c>
-      <c r="G49" s="23" t="s">
-        <v>257</v>
-      </c>
-      <c r="H49" s="22" t="s">
-        <v>283</v>
-      </c>
-      <c r="I49" s="23" t="s">
-        <v>329</v>
-      </c>
-      <c r="J49" s="22">
+      <c r="D49" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E49" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="F49" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="G49" s="22" t="s">
+        <v>255</v>
+      </c>
+      <c r="H49" s="21" t="s">
+        <v>281</v>
+      </c>
+      <c r="I49" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="J49" s="21">
         <v>2</v>
       </c>
-      <c r="K49" s="21" t="s">
-        <v>356</v>
+      <c r="K49" s="20" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="15.75" thickBot="1">
@@ -3231,22 +3231,22 @@
         <v>21</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E50" s="10" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H50" s="9" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I50" s="10" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="J50" s="9">
         <v>1</v>
@@ -3262,29 +3262,29 @@
       <c r="C51" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D51" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="E51" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="F51" s="22" t="s">
-        <v>202</v>
-      </c>
-      <c r="G51" s="23" t="s">
-        <v>254</v>
-      </c>
-      <c r="H51" s="22" t="s">
-        <v>303</v>
-      </c>
-      <c r="I51" s="23" t="s">
-        <v>329</v>
-      </c>
-      <c r="J51" s="22">
-        <v>1</v>
-      </c>
-      <c r="K51" s="21" t="s">
-        <v>356</v>
+      <c r="D51" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="E51" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="F51" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="G51" s="22" t="s">
+        <v>252</v>
+      </c>
+      <c r="H51" s="21" t="s">
+        <v>301</v>
+      </c>
+      <c r="I51" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="J51" s="21">
+        <v>1</v>
+      </c>
+      <c r="K51" s="20" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="52" spans="1:11" ht="15.75" thickBot="1">
@@ -3297,22 +3297,22 @@
         <v>21</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E52" s="10" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="F52" s="9" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G52" s="10" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="H52" s="9" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="J52" s="9">
         <v>1</v>
@@ -3329,22 +3329,22 @@
         <v>21</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E53" s="8" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="F53" s="7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="H53" s="7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I53" s="8" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="J53" s="7">
         <v>4</v>
@@ -3361,22 +3361,22 @@
         <v>21</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E54" s="10" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G54" s="10" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="H54" s="9" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I54" s="10" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="J54" s="9">
         <v>1</v>
@@ -3393,22 +3393,22 @@
         <v>21</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E55" s="8" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F55" s="7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G55" s="8" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I55" s="8" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="J55" s="7">
         <v>1</v>
@@ -3425,22 +3425,22 @@
         <v>21</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="F56" s="9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G56" s="10" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="H56" s="9" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I56" s="10" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="J56" s="9">
         <v>1</v>
@@ -3457,22 +3457,22 @@
         <v>22</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E57" s="8" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F57" s="7" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="G57" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="H57" s="7" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I57" s="8" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="J57" s="7">
         <v>3</v>
@@ -3488,29 +3488,29 @@
       <c r="C58" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D58" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="E58" s="23" t="s">
-        <v>157</v>
-      </c>
-      <c r="F58" s="22" t="s">
-        <v>202</v>
-      </c>
-      <c r="G58" s="23" t="s">
-        <v>264</v>
-      </c>
-      <c r="H58" s="22" t="s">
-        <v>283</v>
-      </c>
-      <c r="I58" s="23" t="s">
-        <v>329</v>
-      </c>
-      <c r="J58" s="22">
-        <v>1</v>
-      </c>
-      <c r="K58" s="21" t="s">
-        <v>356</v>
+      <c r="D58" s="21" t="s">
+        <v>82</v>
+      </c>
+      <c r="E58" s="22" t="s">
+        <v>155</v>
+      </c>
+      <c r="F58" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="G58" s="22" t="s">
+        <v>262</v>
+      </c>
+      <c r="H58" s="21" t="s">
+        <v>281</v>
+      </c>
+      <c r="I58" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="J58" s="21">
+        <v>1</v>
+      </c>
+      <c r="K58" s="20" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="59" spans="1:11" ht="24.75" thickBot="1">
@@ -3523,22 +3523,22 @@
         <v>21</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E59" s="8" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="F59" s="7" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="H59" s="7" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="I59" s="8" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="J59" s="7">
         <v>1</v>
@@ -3555,22 +3555,22 @@
         <v>21</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E60" s="10" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F60" s="9" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="G60" s="10" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="H60" s="9" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="I60" s="10" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="J60" s="9">
         <v>1</v>
@@ -3587,22 +3587,22 @@
         <v>21</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E61" s="8" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F61" s="7" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="G61" s="8" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H61" s="7" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="I61" s="8" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="J61" s="7">
         <v>1</v>
@@ -3618,29 +3618,29 @@
       <c r="C62" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="D62" s="22" t="s">
-        <v>88</v>
-      </c>
-      <c r="E62" s="23" t="s">
-        <v>161</v>
-      </c>
-      <c r="F62" s="22" t="s">
-        <v>205</v>
-      </c>
-      <c r="G62" s="23" t="s">
-        <v>205</v>
-      </c>
-      <c r="H62" s="22" t="s">
-        <v>306</v>
-      </c>
-      <c r="I62" s="23" t="s">
-        <v>329</v>
-      </c>
-      <c r="J62" s="22">
-        <v>1</v>
-      </c>
-      <c r="K62" s="21" t="s">
-        <v>356</v>
+      <c r="D62" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="E62" s="22" t="s">
+        <v>159</v>
+      </c>
+      <c r="F62" s="21" t="s">
+        <v>203</v>
+      </c>
+      <c r="G62" s="22" t="s">
+        <v>203</v>
+      </c>
+      <c r="H62" s="21" t="s">
+        <v>304</v>
+      </c>
+      <c r="I62" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="J62" s="21">
+        <v>1</v>
+      </c>
+      <c r="K62" s="20" t="s">
+        <v>354</v>
       </c>
     </row>
     <row r="63" spans="1:11" ht="36.75" thickBot="1">
@@ -3653,22 +3653,22 @@
         <v>23</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E63" s="8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F63" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="G63" s="8" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="H63" s="7" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="I63" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J63" s="7">
         <v>2</v>
@@ -3685,22 +3685,22 @@
         <v>24</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E64" s="10" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F64" s="9" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="G64" s="10" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="H64" s="9" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="I64" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J64" s="9">
         <v>1</v>
@@ -3717,22 +3717,22 @@
         <v>24</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E65" s="8" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="F65" s="7" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H65" s="7" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="I65" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J65" s="7">
         <v>1</v>
@@ -3749,22 +3749,22 @@
         <v>24</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E66" s="10" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="F66" s="9" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="G66" s="10" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="H66" s="9" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="I66" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J66" s="9">
         <v>1</v>
@@ -3781,22 +3781,22 @@
         <v>24</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E67" s="8" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F67" s="7" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="G67" s="8" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="H67" s="7" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="I67" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J67" s="7">
         <v>1</v>
@@ -3813,22 +3813,22 @@
         <v>25</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E68" s="10" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="F68" s="9" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="G68" s="10" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="H68" s="9" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="I68" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J68" s="9">
         <v>4</v>
@@ -3845,20 +3845,20 @@
         <v>26</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E69" s="8" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="F69" s="7" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="G69" s="8" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="H69" s="7"/>
       <c r="I69" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J69" s="7">
         <v>1</v>
@@ -3875,22 +3875,22 @@
         <v>24</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E70" s="10" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="F70" s="9" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="G70" s="10" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="H70" s="9" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="I70" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J70" s="9">
         <v>1</v>
@@ -3907,22 +3907,22 @@
         <v>24</v>
       </c>
       <c r="D71" s="7" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E71" s="8" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="F71" s="7" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="G71" s="8" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="H71" s="7" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="I71" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J71" s="7">
         <v>1</v>
@@ -3939,22 +3939,22 @@
         <v>24</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E72" s="10" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="F72" s="9" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="G72" s="10" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="H72" s="9" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="I72" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J72" s="9">
         <v>1</v>
@@ -3971,22 +3971,22 @@
         <v>24</v>
       </c>
       <c r="D73" s="7" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E73" s="8" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="F73" s="7" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="G73" s="8" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="H73" s="7" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="I73" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J73" s="7">
         <v>1</v>
@@ -4003,22 +4003,22 @@
         <v>24</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E74" s="10" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="F74" s="9" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="G74" s="10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="H74" s="9" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="I74" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J74" s="9">
         <v>1</v>
@@ -4035,22 +4035,22 @@
         <v>24</v>
       </c>
       <c r="D75" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E75" s="8" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F75" s="7" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="G75" s="8" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="H75" s="7" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="I75" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J75" s="7">
         <v>1</v>
@@ -4067,22 +4067,22 @@
         <v>24</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="E76" s="10" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="F76" s="9" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="G76" s="10" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="H76" s="9" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="I76" s="8" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J76" s="9">
         <v>1</v>
@@ -4099,22 +4099,22 @@
         <v>27</v>
       </c>
       <c r="D77" s="7" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E77" s="8" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="F77" s="7" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="G77" s="8" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="H77" s="7" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="I77" s="8" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="J77" s="7">
         <v>1</v>
@@ -4131,22 +4131,22 @@
         <v>27</v>
       </c>
       <c r="D78" s="9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E78" s="10" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="F78" s="9" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="G78" s="10" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="H78" s="9" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="I78" s="10" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="J78" s="9">
         <v>1</v>
@@ -4154,35 +4154,35 @@
       <c r="K78" s="9"/>
     </row>
     <row r="79" spans="1:11" ht="15.75" thickBot="1">
-      <c r="B79" s="17">
+      <c r="B79" s="16">
         <f t="shared" ref="B79" si="1">ROW(B79)-ROW($B$2)</f>
         <v>77</v>
       </c>
-      <c r="C79" s="18" t="s">
+      <c r="C79" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="D79" s="18" t="s">
+        <v>350</v>
+      </c>
+      <c r="E79" s="19" t="s">
         <v>351</v>
       </c>
-      <c r="D79" s="19" t="s">
+      <c r="F79" s="18" t="s">
+        <v>350</v>
+      </c>
+      <c r="G79" s="19" t="s">
         <v>352</v>
       </c>
-      <c r="E79" s="20" t="s">
-        <v>353</v>
-      </c>
-      <c r="F79" s="19" t="s">
-        <v>352</v>
-      </c>
-      <c r="G79" s="20" t="s">
-        <v>354</v>
-      </c>
-      <c r="H79" s="19" t="s">
-        <v>352</v>
-      </c>
-      <c r="I79" s="20" t="s">
-        <v>352</v>
-      </c>
-      <c r="J79" s="19">
-        <v>1</v>
-      </c>
-      <c r="K79" s="19"/>
+      <c r="H79" s="18" t="s">
+        <v>350</v>
+      </c>
+      <c r="I79" s="19" t="s">
+        <v>350</v>
+      </c>
+      <c r="J79" s="18">
+        <v>1</v>
+      </c>
+      <c r="K79" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>